<commit_message>
Adiciona telas do simulador ao README e ajusta formatação da planilha
Prints do Resumo, Comparativo RET, Transição, Premissas e DRE em docs/.
Na planilha: anos sem separador de milhar, rótulos encurtados para não
cortar e alinhamento da tabela de transição.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNUG9G5PiaxGmiV8dk6CnD
</commit_message>
<xml_diff>
--- a/simulador_reforma_tributaria_imoveis_v4.xlsx
+++ b/simulador_reforma_tributaria_imoveis_v4.xlsx
@@ -374,7 +374,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -725,6 +725,9 @@
     <xf numFmtId="164" fontId="22" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="22" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -738,24 +741,56 @@
     <xf numFmtId="165" fontId="24" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="12" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="15" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="23" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="13" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="24" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="13" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -6176,7 +6211,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Versão consultiva v4</t>
+          <t>Versão v4</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -6330,7 +6365,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Tributos no ciclo — RET (art. 485)</t>
+          <t>Tributos no ciclo — RET</t>
         </is>
       </c>
       <c r="G18" s="115">
@@ -6809,12 +6844,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="150" t="inlineStr">
+      <c r="A9" s="161" t="inlineStr">
         <is>
           <t>Check vs. Premissas</t>
         </is>
       </c>
-      <c r="B9" s="151">
+      <c r="B9" s="162">
         <f>ROUND(B8-'Premissas &amp; Cenários'!$E$102,2)</f>
         <v/>
       </c>
@@ -11043,7 +11078,7 @@
     <row r="91">
       <c r="A91" s="123" t="inlineStr">
         <is>
-          <t>Serviços de construção e mão de obra terceirizados — crédito à alíquota reduzida (art. 261)</t>
+          <t>Obra terceirizada (serviços e mão de obra) — crédito reduzido</t>
         </is>
       </c>
       <c r="B91" s="124" t="n">
@@ -11283,7 +11318,7 @@
     <row r="105">
       <c r="A105" s="123" t="inlineStr">
         <is>
-          <t>Aplicar LC 224/2025 (presunção +10% sobre receita acima de R$ 5 mi/ano)?</t>
+          <t>Aplicar a majoração da LC 224/2025?</t>
         </is>
       </c>
       <c r="B105" s="130" t="inlineStr">
@@ -12084,7 +12119,7 @@
         <f>SUM($D$43:D43)</f>
         <v/>
       </c>
-      <c r="N43" s="44">
+      <c r="N43" s="134">
         <f>IF(A43&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A43&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A43&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A43&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12173,7 +12208,7 @@
         <f>SUM($D$43:D44)</f>
         <v/>
       </c>
-      <c r="N44" s="44">
+      <c r="N44" s="134">
         <f>IF(A44&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A44&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A44&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A44&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12262,7 +12297,7 @@
         <f>SUM($D$43:D45)</f>
         <v/>
       </c>
-      <c r="N45" s="44">
+      <c r="N45" s="134">
         <f>IF(A45&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A45&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A45&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A45&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12351,7 +12386,7 @@
         <f>SUM($D$43:D46)</f>
         <v/>
       </c>
-      <c r="N46" s="44">
+      <c r="N46" s="134">
         <f>IF(A46&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A46&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A46&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A46&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12440,7 +12475,7 @@
         <f>SUM($D$43:D47)</f>
         <v/>
       </c>
-      <c r="N47" s="44">
+      <c r="N47" s="134">
         <f>IF(A47&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A47&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A47&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A47&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12529,7 +12564,7 @@
         <f>SUM($D$43:D48)</f>
         <v/>
       </c>
-      <c r="N48" s="44">
+      <c r="N48" s="134">
         <f>IF(A48&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A48&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A48&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A48&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12618,7 +12653,7 @@
         <f>SUM($D$43:D49)</f>
         <v/>
       </c>
-      <c r="N49" s="44">
+      <c r="N49" s="134">
         <f>IF(A49&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A49&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A49&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A49&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12707,7 +12742,7 @@
         <f>SUM($D$43:D50)</f>
         <v/>
       </c>
-      <c r="N50" s="44">
+      <c r="N50" s="134">
         <f>IF(A50&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A50&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A50&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A50&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12796,7 +12831,7 @@
         <f>SUM($D$43:D51)</f>
         <v/>
       </c>
-      <c r="N51" s="44">
+      <c r="N51" s="134">
         <f>IF(A51&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A51&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A51&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A51&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12885,7 +12920,7 @@
         <f>SUM($D$43:D52)</f>
         <v/>
       </c>
-      <c r="N52" s="44">
+      <c r="N52" s="134">
         <f>IF(A52&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A52&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A52&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A52&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -12974,7 +13009,7 @@
         <f>SUM($D$43:D53)</f>
         <v/>
       </c>
-      <c r="N53" s="44">
+      <c r="N53" s="134">
         <f>IF(A53&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A53&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A53&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A53&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13063,7 +13098,7 @@
         <f>SUM($D$43:D54)</f>
         <v/>
       </c>
-      <c r="N54" s="44">
+      <c r="N54" s="134">
         <f>IF(A54&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A54&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A54&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A54&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13152,7 +13187,7 @@
         <f>SUM($D$43:D55)</f>
         <v/>
       </c>
-      <c r="N55" s="44">
+      <c r="N55" s="134">
         <f>IF(A55&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A55&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A55&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A55&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13241,7 +13276,7 @@
         <f>SUM($D$43:D56)</f>
         <v/>
       </c>
-      <c r="N56" s="44">
+      <c r="N56" s="134">
         <f>IF(A56&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A56&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A56&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A56&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13330,7 +13365,7 @@
         <f>SUM($D$43:D57)</f>
         <v/>
       </c>
-      <c r="N57" s="44">
+      <c r="N57" s="134">
         <f>IF(A57&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A57&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A57&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A57&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13419,7 +13454,7 @@
         <f>SUM($D$43:D58)</f>
         <v/>
       </c>
-      <c r="N58" s="44">
+      <c r="N58" s="134">
         <f>IF(A58&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A58&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A58&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A58&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13508,7 +13543,7 @@
         <f>SUM($D$43:D59)</f>
         <v/>
       </c>
-      <c r="N59" s="44">
+      <c r="N59" s="134">
         <f>IF(A59&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A59&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A59&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A59&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13597,7 +13632,7 @@
         <f>SUM($D$43:D60)</f>
         <v/>
       </c>
-      <c r="N60" s="44">
+      <c r="N60" s="134">
         <f>IF(A60&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A60&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A60&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A60&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13686,7 +13721,7 @@
         <f>SUM($D$43:D61)</f>
         <v/>
       </c>
-      <c r="N61" s="44">
+      <c r="N61" s="134">
         <f>IF(A61&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A61&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A61&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A61&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13775,7 +13810,7 @@
         <f>SUM($D$43:D62)</f>
         <v/>
       </c>
-      <c r="N62" s="44">
+      <c r="N62" s="134">
         <f>IF(A62&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A62&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A62&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A62&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13864,7 +13899,7 @@
         <f>SUM($D$43:D63)</f>
         <v/>
       </c>
-      <c r="N63" s="44">
+      <c r="N63" s="134">
         <f>IF(A63&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A63&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A63&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A63&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -13953,7 +13988,7 @@
         <f>SUM($D$43:D64)</f>
         <v/>
       </c>
-      <c r="N64" s="44">
+      <c r="N64" s="134">
         <f>IF(A64&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A64&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A64&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A64&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14042,7 +14077,7 @@
         <f>SUM($D$43:D65)</f>
         <v/>
       </c>
-      <c r="N65" s="44">
+      <c r="N65" s="134">
         <f>IF(A65&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A65&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A65&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A65&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14131,7 +14166,7 @@
         <f>SUM($D$43:D66)</f>
         <v/>
       </c>
-      <c r="N66" s="44">
+      <c r="N66" s="134">
         <f>IF(A66&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A66&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A66&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A66&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14220,7 +14255,7 @@
         <f>SUM($D$43:D67)</f>
         <v/>
       </c>
-      <c r="N67" s="44">
+      <c r="N67" s="134">
         <f>IF(A67&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A67&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A67&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A67&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14309,7 +14344,7 @@
         <f>SUM($D$43:D68)</f>
         <v/>
       </c>
-      <c r="N68" s="44">
+      <c r="N68" s="134">
         <f>IF(A68&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A68&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A68&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A68&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14398,7 +14433,7 @@
         <f>SUM($D$43:D69)</f>
         <v/>
       </c>
-      <c r="N69" s="44">
+      <c r="N69" s="134">
         <f>IF(A69&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A69&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A69&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A69&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14487,7 +14522,7 @@
         <f>SUM($D$43:D70)</f>
         <v/>
       </c>
-      <c r="N70" s="44">
+      <c r="N70" s="134">
         <f>IF(A70&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A70&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A70&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A70&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14576,7 +14611,7 @@
         <f>SUM($D$43:D71)</f>
         <v/>
       </c>
-      <c r="N71" s="44">
+      <c r="N71" s="134">
         <f>IF(A71&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A71&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A71&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A71&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14665,7 +14700,7 @@
         <f>SUM($D$43:D72)</f>
         <v/>
       </c>
-      <c r="N72" s="44">
+      <c r="N72" s="134">
         <f>IF(A72&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A72&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A72&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A72&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14754,7 +14789,7 @@
         <f>SUM($D$43:D73)</f>
         <v/>
       </c>
-      <c r="N73" s="44">
+      <c r="N73" s="134">
         <f>IF(A73&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A73&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A73&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A73&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14843,7 +14878,7 @@
         <f>SUM($D$43:D74)</f>
         <v/>
       </c>
-      <c r="N74" s="44">
+      <c r="N74" s="134">
         <f>IF(A74&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A74&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A74&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A74&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -14932,7 +14967,7 @@
         <f>SUM($D$43:D75)</f>
         <v/>
       </c>
-      <c r="N75" s="44">
+      <c r="N75" s="134">
         <f>IF(A75&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A75&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A75&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A75&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15021,7 +15056,7 @@
         <f>SUM($D$43:D76)</f>
         <v/>
       </c>
-      <c r="N76" s="44">
+      <c r="N76" s="134">
         <f>IF(A76&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A76&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A76&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A76&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15110,7 +15145,7 @@
         <f>SUM($D$43:D77)</f>
         <v/>
       </c>
-      <c r="N77" s="44">
+      <c r="N77" s="134">
         <f>IF(A77&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A77&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A77&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A77&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15199,7 +15234,7 @@
         <f>SUM($D$43:D78)</f>
         <v/>
       </c>
-      <c r="N78" s="44">
+      <c r="N78" s="134">
         <f>IF(A78&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A78&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A78&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A78&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15288,7 +15323,7 @@
         <f>SUM($D$43:D79)</f>
         <v/>
       </c>
-      <c r="N79" s="44">
+      <c r="N79" s="134">
         <f>IF(A79&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A79&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A79&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A79&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15377,7 +15412,7 @@
         <f>SUM($D$43:D80)</f>
         <v/>
       </c>
-      <c r="N80" s="44">
+      <c r="N80" s="134">
         <f>IF(A80&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A80&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A80&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A80&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15466,7 +15501,7 @@
         <f>SUM($D$43:D81)</f>
         <v/>
       </c>
-      <c r="N81" s="44">
+      <c r="N81" s="134">
         <f>IF(A81&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A81&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A81&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A81&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15555,7 +15590,7 @@
         <f>SUM($D$43:D82)</f>
         <v/>
       </c>
-      <c r="N82" s="44">
+      <c r="N82" s="134">
         <f>IF(A82&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A82&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A82&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A82&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15644,7 +15679,7 @@
         <f>SUM($D$43:D83)</f>
         <v/>
       </c>
-      <c r="N83" s="44">
+      <c r="N83" s="134">
         <f>IF(A83&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A83&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A83&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A83&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15733,7 +15768,7 @@
         <f>SUM($D$43:D84)</f>
         <v/>
       </c>
-      <c r="N84" s="44">
+      <c r="N84" s="134">
         <f>IF(A84&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A84&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A84&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A84&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15822,7 +15857,7 @@
         <f>SUM($D$43:D85)</f>
         <v/>
       </c>
-      <c r="N85" s="44">
+      <c r="N85" s="134">
         <f>IF(A85&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A85&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A85&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A85&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -15911,7 +15946,7 @@
         <f>SUM($D$43:D86)</f>
         <v/>
       </c>
-      <c r="N86" s="44">
+      <c r="N86" s="134">
         <f>IF(A86&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A86&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A86&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A86&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16000,7 +16035,7 @@
         <f>SUM($D$43:D87)</f>
         <v/>
       </c>
-      <c r="N87" s="44">
+      <c r="N87" s="134">
         <f>IF(A87&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A87&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A87&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A87&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16089,7 +16124,7 @@
         <f>SUM($D$43:D88)</f>
         <v/>
       </c>
-      <c r="N88" s="44">
+      <c r="N88" s="134">
         <f>IF(A88&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A88&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A88&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A88&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16178,7 +16213,7 @@
         <f>SUM($D$43:D89)</f>
         <v/>
       </c>
-      <c r="N89" s="44">
+      <c r="N89" s="134">
         <f>IF(A89&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A89&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A89&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A89&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16267,7 +16302,7 @@
         <f>SUM($D$43:D90)</f>
         <v/>
       </c>
-      <c r="N90" s="44">
+      <c r="N90" s="134">
         <f>IF(A90&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A90&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A90&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A90&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16356,7 +16391,7 @@
         <f>SUM($D$43:D91)</f>
         <v/>
       </c>
-      <c r="N91" s="44">
+      <c r="N91" s="134">
         <f>IF(A91&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A91&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A91&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A91&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16445,7 +16480,7 @@
         <f>SUM($D$43:D92)</f>
         <v/>
       </c>
-      <c r="N92" s="44">
+      <c r="N92" s="134">
         <f>IF(A92&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A92&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A92&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A92&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16534,7 +16569,7 @@
         <f>SUM($D$43:D93)</f>
         <v/>
       </c>
-      <c r="N93" s="44">
+      <c r="N93" s="134">
         <f>IF(A93&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A93&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A93&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A93&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16623,7 +16658,7 @@
         <f>SUM($D$43:D94)</f>
         <v/>
       </c>
-      <c r="N94" s="44">
+      <c r="N94" s="134">
         <f>IF(A94&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A94&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A94&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A94&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16712,7 +16747,7 @@
         <f>SUM($D$43:D95)</f>
         <v/>
       </c>
-      <c r="N95" s="44">
+      <c r="N95" s="134">
         <f>IF(A95&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A95&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A95&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A95&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16801,7 +16836,7 @@
         <f>SUM($D$43:D96)</f>
         <v/>
       </c>
-      <c r="N96" s="44">
+      <c r="N96" s="134">
         <f>IF(A96&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A96&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A96&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A96&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16890,7 +16925,7 @@
         <f>SUM($D$43:D97)</f>
         <v/>
       </c>
-      <c r="N97" s="44">
+      <c r="N97" s="134">
         <f>IF(A97&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A97&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A97&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A97&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -16979,7 +17014,7 @@
         <f>SUM($D$43:D98)</f>
         <v/>
       </c>
-      <c r="N98" s="44">
+      <c r="N98" s="134">
         <f>IF(A98&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A98&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A98&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A98&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -17068,7 +17103,7 @@
         <f>SUM($D$43:D99)</f>
         <v/>
       </c>
-      <c r="N99" s="44">
+      <c r="N99" s="134">
         <f>IF(A99&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A99&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A99&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A99&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -17157,7 +17192,7 @@
         <f>SUM($D$43:D100)</f>
         <v/>
       </c>
-      <c r="N100" s="44">
+      <c r="N100" s="134">
         <f>IF(A100&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A100&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A100&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A100&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -17246,7 +17281,7 @@
         <f>SUM($D$43:D101)</f>
         <v/>
       </c>
-      <c r="N101" s="44">
+      <c r="N101" s="134">
         <f>IF(A101&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A101&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A101&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A101&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -17335,7 +17370,7 @@
         <f>SUM($D$43:D102)</f>
         <v/>
       </c>
-      <c r="N102" s="44">
+      <c r="N102" s="134">
         <f>IF(A102&lt;=12,'Premissas &amp; Cenários'!$B$50,IF(A102&lt;=24,'Premissas &amp; Cenários'!$B$50+1,IF(A102&lt;=36,'Premissas &amp; Cenários'!$B$50+2,IF(A102&lt;=48,'Premissas &amp; Cenários'!$B$50+3,'Premissas &amp; Cenários'!$B$50+4))))</f>
         <v/>
       </c>
@@ -17563,7 +17598,7 @@
   <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
-    <col width="31.85546875" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
   </cols>
@@ -17602,7 +17637,7 @@
           <t>DRE consolidada por cenário</t>
         </is>
       </c>
-      <c r="B6" s="134">
+      <c r="B6" s="135">
         <f>"Todas as colunas no modo: "&amp;'Matriz Normativa &amp; Governança'!$C$8&amp;" (selecionado na aba Matriz Normativa &amp; Governança)"</f>
         <v/>
       </c>
@@ -18075,19 +18110,19 @@
           <t>Base de presunção IRPJ (com LC 224)</t>
         </is>
       </c>
-      <c r="B25" s="135">
+      <c r="B25" s="136">
         <f>'IRPJ_CSLL Trimestral'!$I$27</f>
         <v/>
       </c>
-      <c r="C25" s="135">
+      <c r="C25" s="136">
         <f>'IRPJ_CSLL Trimestral'!$I$27</f>
         <v/>
       </c>
-      <c r="D25" s="135">
+      <c r="D25" s="136">
         <f>'IRPJ_CSLL Trimestral'!$I$27</f>
         <v/>
       </c>
-      <c r="E25" s="136">
+      <c r="E25" s="137">
         <f>'IRPJ_CSLL Trimestral'!$I$27</f>
         <v/>
       </c>
@@ -18103,19 +18138,19 @@
           <t>IRPJ básico</t>
         </is>
       </c>
-      <c r="B26" s="135">
+      <c r="B26" s="136">
         <f>'IRPJ_CSLL Trimestral'!$J$27</f>
         <v/>
       </c>
-      <c r="C26" s="135">
+      <c r="C26" s="136">
         <f>'IRPJ_CSLL Trimestral'!$J$27</f>
         <v/>
       </c>
-      <c r="D26" s="135">
+      <c r="D26" s="136">
         <f>'IRPJ_CSLL Trimestral'!$J$27</f>
         <v/>
       </c>
-      <c r="E26" s="136">
+      <c r="E26" s="137">
         <f>'IRPJ_CSLL Trimestral'!$J$27</f>
         <v/>
       </c>
@@ -18131,19 +18166,19 @@
           <t>IRPJ adicional</t>
         </is>
       </c>
-      <c r="B27" s="137">
+      <c r="B27" s="138">
         <f>'IRPJ_CSLL Trimestral'!$K$27</f>
         <v/>
       </c>
-      <c r="C27" s="137">
+      <c r="C27" s="138">
         <f>'IRPJ_CSLL Trimestral'!$K$27</f>
         <v/>
       </c>
-      <c r="D27" s="137">
+      <c r="D27" s="138">
         <f>'IRPJ_CSLL Trimestral'!$K$27</f>
         <v/>
       </c>
-      <c r="E27" s="138">
+      <c r="E27" s="139">
         <f>'IRPJ_CSLL Trimestral'!$K$27</f>
         <v/>
       </c>
@@ -18159,19 +18194,19 @@
           <t>Base de presunção CSLL (com LC 224)</t>
         </is>
       </c>
-      <c r="B28" s="135">
+      <c r="B28" s="136">
         <f>'IRPJ_CSLL Trimestral'!$L$27</f>
         <v/>
       </c>
-      <c r="C28" s="135">
+      <c r="C28" s="136">
         <f>'IRPJ_CSLL Trimestral'!$L$27</f>
         <v/>
       </c>
-      <c r="D28" s="135">
+      <c r="D28" s="136">
         <f>'IRPJ_CSLL Trimestral'!$L$27</f>
         <v/>
       </c>
-      <c r="E28" s="136">
+      <c r="E28" s="137">
         <f>'IRPJ_CSLL Trimestral'!$L$27</f>
         <v/>
       </c>
@@ -18187,19 +18222,19 @@
           <t>CSLL</t>
         </is>
       </c>
-      <c r="B29" s="135">
+      <c r="B29" s="136">
         <f>'IRPJ_CSLL Trimestral'!$M$27</f>
         <v/>
       </c>
-      <c r="C29" s="135">
+      <c r="C29" s="136">
         <f>'IRPJ_CSLL Trimestral'!$M$27</f>
         <v/>
       </c>
-      <c r="D29" s="135">
+      <c r="D29" s="136">
         <f>'IRPJ_CSLL Trimestral'!$M$27</f>
         <v/>
       </c>
-      <c r="E29" s="136">
+      <c r="E29" s="137">
         <f>'IRPJ_CSLL Trimestral'!$M$27</f>
         <v/>
       </c>
@@ -18564,23 +18599,23 @@
           <t>Rubrica</t>
         </is>
       </c>
-      <c r="B47" s="76">
+      <c r="B47" s="140">
         <f>'Premissas &amp; Cenários'!$B$50</f>
         <v/>
       </c>
-      <c r="C47" s="76">
+      <c r="C47" s="140">
         <f>B47+1</f>
         <v/>
       </c>
-      <c r="D47" s="76">
+      <c r="D47" s="140">
         <f>C47+1</f>
         <v/>
       </c>
-      <c r="E47" s="76">
+      <c r="E47" s="140">
         <f>D47+1</f>
         <v/>
       </c>
-      <c r="F47" s="76">
+      <c r="F47" s="140">
         <f>E47+1</f>
         <v/>
       </c>
@@ -19123,7 +19158,7 @@
           <t>Receita de vendas (tributável)</t>
         </is>
       </c>
-      <c r="E67" s="139">
+      <c r="E67" s="141">
         <f>E8</f>
         <v/>
       </c>
@@ -19139,7 +19174,7 @@
           <t>Receita de permuta física a valor justo</t>
         </is>
       </c>
-      <c r="E68" s="140">
+      <c r="E68" s="142">
         <f>'Premissas &amp; Cenários'!$G$56</f>
         <v/>
       </c>
@@ -19155,7 +19190,7 @@
           <t>Receita bruta societária</t>
         </is>
       </c>
-      <c r="E69" s="141">
+      <c r="E69" s="143">
         <f>E67+E68</f>
         <v/>
       </c>
@@ -19171,7 +19206,7 @@
           <t>Custo do terreno adquirido por permuta</t>
         </is>
       </c>
-      <c r="E70" s="139">
+      <c r="E70" s="141">
         <f>-E68</f>
         <v/>
       </c>
@@ -19187,7 +19222,7 @@
           <t>Efeito líquido da permuta no lucro</t>
         </is>
       </c>
-      <c r="E71" s="139">
+      <c r="E71" s="141">
         <f>E68+E70</f>
         <v/>
       </c>
@@ -19254,23 +19289,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="142" t="inlineStr">
+      <c r="B1" s="144" t="inlineStr">
         <is>
           <t>IRPJ e CSLL — Lucro Presumido trimestral (LC 224/2025)</t>
         </is>
       </c>
-      <c r="C1" s="143" t="n"/>
-      <c r="D1" s="143" t="n"/>
-      <c r="E1" s="143" t="n"/>
-      <c r="F1" s="143" t="n"/>
-      <c r="G1" s="143" t="n"/>
-      <c r="H1" s="143" t="n"/>
-      <c r="I1" s="143" t="n"/>
-      <c r="J1" s="143" t="n"/>
-      <c r="K1" s="143" t="n"/>
-      <c r="L1" s="143" t="n"/>
-      <c r="M1" s="143" t="n"/>
-      <c r="N1" s="143" t="n"/>
+      <c r="C1" s="145" t="n"/>
+      <c r="D1" s="145" t="n"/>
+      <c r="E1" s="145" t="n"/>
+      <c r="F1" s="145" t="n"/>
+      <c r="G1" s="145" t="n"/>
+      <c r="H1" s="145" t="n"/>
+      <c r="I1" s="145" t="n"/>
+      <c r="J1" s="145" t="n"/>
+      <c r="K1" s="145" t="n"/>
+      <c r="L1" s="145" t="n"/>
+      <c r="M1" s="145" t="n"/>
+      <c r="N1" s="145" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -19364,7 +19399,7 @@
       <c r="A7" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="144">
+      <c r="B7" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A7-1)/4)</f>
         <v/>
       </c>
@@ -19372,47 +19407,47 @@
         <f>MOD(A7-1,4)+1</f>
         <v/>
       </c>
-      <c r="D7" s="140">
+      <c r="D7" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A7)</f>
         <v/>
       </c>
-      <c r="E7" s="139">
+      <c r="E7" s="141">
         <f>IF(C7=1,D7,E6+D7)</f>
         <v/>
       </c>
-      <c r="F7" s="140">
+      <c r="F7" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C7</f>
         <v/>
       </c>
-      <c r="G7" s="139">
+      <c r="G7" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E7-F7),0)</f>
         <v/>
       </c>
-      <c r="H7" s="139">
+      <c r="H7" s="141">
         <f>IF(C7=1,G7,G7-G6)</f>
         <v/>
       </c>
-      <c r="I7" s="139">
+      <c r="I7" s="141">
         <f>MAX(0,D7*'Premissas &amp; Cenários'!$B$44+H7*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J7" s="139">
+      <c r="J7" s="141">
         <f>I7*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K7" s="139">
+      <c r="K7" s="141">
         <f>MAX(0,I7-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L7" s="139">
+      <c r="L7" s="141">
         <f>MAX(0,D7*'Premissas &amp; Cenários'!$B$48+IF(AND(B7=2026,C7=1),0,H7*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M7" s="139">
+      <c r="M7" s="141">
         <f>L7*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N7" s="139">
+      <c r="N7" s="141">
         <f>J7+K7+M7</f>
         <v/>
       </c>
@@ -19421,7 +19456,7 @@
       <c r="A8" s="123" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="144">
+      <c r="B8" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A8-1)/4)</f>
         <v/>
       </c>
@@ -19429,47 +19464,47 @@
         <f>MOD(A8-1,4)+1</f>
         <v/>
       </c>
-      <c r="D8" s="140">
+      <c r="D8" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A8)</f>
         <v/>
       </c>
-      <c r="E8" s="139">
+      <c r="E8" s="141">
         <f>IF(C8=1,D8,E7+D8)</f>
         <v/>
       </c>
-      <c r="F8" s="140">
+      <c r="F8" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C8</f>
         <v/>
       </c>
-      <c r="G8" s="139">
+      <c r="G8" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E8-F8),0)</f>
         <v/>
       </c>
-      <c r="H8" s="139">
+      <c r="H8" s="141">
         <f>IF(C8=1,G8,G8-G7)</f>
         <v/>
       </c>
-      <c r="I8" s="139">
+      <c r="I8" s="141">
         <f>MAX(0,D8*'Premissas &amp; Cenários'!$B$44+H8*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J8" s="139">
+      <c r="J8" s="141">
         <f>I8*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K8" s="139">
+      <c r="K8" s="141">
         <f>MAX(0,I8-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L8" s="139">
+      <c r="L8" s="141">
         <f>MAX(0,D8*'Premissas &amp; Cenários'!$B$48+IF(AND(B8=2026,C8=1),0,H8*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M8" s="139">
+      <c r="M8" s="141">
         <f>L8*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N8" s="139">
+      <c r="N8" s="141">
         <f>J8+K8+M8</f>
         <v/>
       </c>
@@ -19478,7 +19513,7 @@
       <c r="A9" s="123" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="144">
+      <c r="B9" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A9-1)/4)</f>
         <v/>
       </c>
@@ -19486,47 +19521,47 @@
         <f>MOD(A9-1,4)+1</f>
         <v/>
       </c>
-      <c r="D9" s="140">
+      <c r="D9" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A9)</f>
         <v/>
       </c>
-      <c r="E9" s="139">
+      <c r="E9" s="141">
         <f>IF(C9=1,D9,E8+D9)</f>
         <v/>
       </c>
-      <c r="F9" s="140">
+      <c r="F9" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C9</f>
         <v/>
       </c>
-      <c r="G9" s="139">
+      <c r="G9" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E9-F9),0)</f>
         <v/>
       </c>
-      <c r="H9" s="139">
+      <c r="H9" s="141">
         <f>IF(C9=1,G9,G9-G8)</f>
         <v/>
       </c>
-      <c r="I9" s="139">
+      <c r="I9" s="141">
         <f>MAX(0,D9*'Premissas &amp; Cenários'!$B$44+H9*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J9" s="139">
+      <c r="J9" s="141">
         <f>I9*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K9" s="139">
+      <c r="K9" s="141">
         <f>MAX(0,I9-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L9" s="139">
+      <c r="L9" s="141">
         <f>MAX(0,D9*'Premissas &amp; Cenários'!$B$48+IF(AND(B9=2026,C9=1),0,H9*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M9" s="139">
+      <c r="M9" s="141">
         <f>L9*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N9" s="139">
+      <c r="N9" s="141">
         <f>J9+K9+M9</f>
         <v/>
       </c>
@@ -19535,7 +19570,7 @@
       <c r="A10" s="123" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="144">
+      <c r="B10" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A10-1)/4)</f>
         <v/>
       </c>
@@ -19543,47 +19578,47 @@
         <f>MOD(A10-1,4)+1</f>
         <v/>
       </c>
-      <c r="D10" s="140">
+      <c r="D10" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A10)</f>
         <v/>
       </c>
-      <c r="E10" s="139">
+      <c r="E10" s="141">
         <f>IF(C10=1,D10,E9+D10)</f>
         <v/>
       </c>
-      <c r="F10" s="140">
+      <c r="F10" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C10</f>
         <v/>
       </c>
-      <c r="G10" s="139">
+      <c r="G10" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E10-F10),0)</f>
         <v/>
       </c>
-      <c r="H10" s="139">
+      <c r="H10" s="141">
         <f>IF(C10=1,G10,G10-G9)</f>
         <v/>
       </c>
-      <c r="I10" s="139">
+      <c r="I10" s="141">
         <f>MAX(0,D10*'Premissas &amp; Cenários'!$B$44+H10*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J10" s="139">
+      <c r="J10" s="141">
         <f>I10*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K10" s="139">
+      <c r="K10" s="141">
         <f>MAX(0,I10-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L10" s="139">
+      <c r="L10" s="141">
         <f>MAX(0,D10*'Premissas &amp; Cenários'!$B$48+IF(AND(B10=2026,C10=1),0,H10*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M10" s="139">
+      <c r="M10" s="141">
         <f>L10*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N10" s="139">
+      <c r="N10" s="141">
         <f>J10+K10+M10</f>
         <v/>
       </c>
@@ -19592,7 +19627,7 @@
       <c r="A11" s="123" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="144">
+      <c r="B11" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A11-1)/4)</f>
         <v/>
       </c>
@@ -19600,47 +19635,47 @@
         <f>MOD(A11-1,4)+1</f>
         <v/>
       </c>
-      <c r="D11" s="140">
+      <c r="D11" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A11)</f>
         <v/>
       </c>
-      <c r="E11" s="139">
+      <c r="E11" s="141">
         <f>IF(C11=1,D11,E10+D11)</f>
         <v/>
       </c>
-      <c r="F11" s="140">
+      <c r="F11" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C11</f>
         <v/>
       </c>
-      <c r="G11" s="139">
+      <c r="G11" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E11-F11),0)</f>
         <v/>
       </c>
-      <c r="H11" s="139">
+      <c r="H11" s="141">
         <f>IF(C11=1,G11,G11-G10)</f>
         <v/>
       </c>
-      <c r="I11" s="139">
+      <c r="I11" s="141">
         <f>MAX(0,D11*'Premissas &amp; Cenários'!$B$44+H11*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J11" s="139">
+      <c r="J11" s="141">
         <f>I11*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K11" s="139">
+      <c r="K11" s="141">
         <f>MAX(0,I11-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L11" s="139">
+      <c r="L11" s="141">
         <f>MAX(0,D11*'Premissas &amp; Cenários'!$B$48+IF(AND(B11=2026,C11=1),0,H11*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M11" s="139">
+      <c r="M11" s="141">
         <f>L11*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N11" s="139">
+      <c r="N11" s="141">
         <f>J11+K11+M11</f>
         <v/>
       </c>
@@ -19649,7 +19684,7 @@
       <c r="A12" s="123" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="144">
+      <c r="B12" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A12-1)/4)</f>
         <v/>
       </c>
@@ -19657,47 +19692,47 @@
         <f>MOD(A12-1,4)+1</f>
         <v/>
       </c>
-      <c r="D12" s="140">
+      <c r="D12" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A12)</f>
         <v/>
       </c>
-      <c r="E12" s="139">
+      <c r="E12" s="141">
         <f>IF(C12=1,D12,E11+D12)</f>
         <v/>
       </c>
-      <c r="F12" s="140">
+      <c r="F12" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C12</f>
         <v/>
       </c>
-      <c r="G12" s="139">
+      <c r="G12" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E12-F12),0)</f>
         <v/>
       </c>
-      <c r="H12" s="139">
+      <c r="H12" s="141">
         <f>IF(C12=1,G12,G12-G11)</f>
         <v/>
       </c>
-      <c r="I12" s="139">
+      <c r="I12" s="141">
         <f>MAX(0,D12*'Premissas &amp; Cenários'!$B$44+H12*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J12" s="139">
+      <c r="J12" s="141">
         <f>I12*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K12" s="139">
+      <c r="K12" s="141">
         <f>MAX(0,I12-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L12" s="139">
+      <c r="L12" s="141">
         <f>MAX(0,D12*'Premissas &amp; Cenários'!$B$48+IF(AND(B12=2026,C12=1),0,H12*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M12" s="139">
+      <c r="M12" s="141">
         <f>L12*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N12" s="139">
+      <c r="N12" s="141">
         <f>J12+K12+M12</f>
         <v/>
       </c>
@@ -19706,7 +19741,7 @@
       <c r="A13" s="123" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="144">
+      <c r="B13" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A13-1)/4)</f>
         <v/>
       </c>
@@ -19714,47 +19749,47 @@
         <f>MOD(A13-1,4)+1</f>
         <v/>
       </c>
-      <c r="D13" s="140">
+      <c r="D13" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A13)</f>
         <v/>
       </c>
-      <c r="E13" s="139">
+      <c r="E13" s="141">
         <f>IF(C13=1,D13,E12+D13)</f>
         <v/>
       </c>
-      <c r="F13" s="140">
+      <c r="F13" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C13</f>
         <v/>
       </c>
-      <c r="G13" s="139">
+      <c r="G13" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E13-F13),0)</f>
         <v/>
       </c>
-      <c r="H13" s="139">
+      <c r="H13" s="141">
         <f>IF(C13=1,G13,G13-G12)</f>
         <v/>
       </c>
-      <c r="I13" s="139">
+      <c r="I13" s="141">
         <f>MAX(0,D13*'Premissas &amp; Cenários'!$B$44+H13*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J13" s="139">
+      <c r="J13" s="141">
         <f>I13*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K13" s="139">
+      <c r="K13" s="141">
         <f>MAX(0,I13-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L13" s="139">
+      <c r="L13" s="141">
         <f>MAX(0,D13*'Premissas &amp; Cenários'!$B$48+IF(AND(B13=2026,C13=1),0,H13*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M13" s="139">
+      <c r="M13" s="141">
         <f>L13*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N13" s="139">
+      <c r="N13" s="141">
         <f>J13+K13+M13</f>
         <v/>
       </c>
@@ -19763,7 +19798,7 @@
       <c r="A14" s="123" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="144">
+      <c r="B14" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A14-1)/4)</f>
         <v/>
       </c>
@@ -19771,47 +19806,47 @@
         <f>MOD(A14-1,4)+1</f>
         <v/>
       </c>
-      <c r="D14" s="140">
+      <c r="D14" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A14)</f>
         <v/>
       </c>
-      <c r="E14" s="139">
+      <c r="E14" s="141">
         <f>IF(C14=1,D14,E13+D14)</f>
         <v/>
       </c>
-      <c r="F14" s="140">
+      <c r="F14" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C14</f>
         <v/>
       </c>
-      <c r="G14" s="139">
+      <c r="G14" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E14-F14),0)</f>
         <v/>
       </c>
-      <c r="H14" s="139">
+      <c r="H14" s="141">
         <f>IF(C14=1,G14,G14-G13)</f>
         <v/>
       </c>
-      <c r="I14" s="139">
+      <c r="I14" s="141">
         <f>MAX(0,D14*'Premissas &amp; Cenários'!$B$44+H14*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J14" s="139">
+      <c r="J14" s="141">
         <f>I14*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K14" s="139">
+      <c r="K14" s="141">
         <f>MAX(0,I14-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L14" s="139">
+      <c r="L14" s="141">
         <f>MAX(0,D14*'Premissas &amp; Cenários'!$B$48+IF(AND(B14=2026,C14=1),0,H14*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M14" s="139">
+      <c r="M14" s="141">
         <f>L14*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N14" s="139">
+      <c r="N14" s="141">
         <f>J14+K14+M14</f>
         <v/>
       </c>
@@ -19820,7 +19855,7 @@
       <c r="A15" s="123" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="144">
+      <c r="B15" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A15-1)/4)</f>
         <v/>
       </c>
@@ -19828,47 +19863,47 @@
         <f>MOD(A15-1,4)+1</f>
         <v/>
       </c>
-      <c r="D15" s="140">
+      <c r="D15" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A15)</f>
         <v/>
       </c>
-      <c r="E15" s="139">
+      <c r="E15" s="141">
         <f>IF(C15=1,D15,E14+D15)</f>
         <v/>
       </c>
-      <c r="F15" s="140">
+      <c r="F15" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C15</f>
         <v/>
       </c>
-      <c r="G15" s="139">
+      <c r="G15" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E15-F15),0)</f>
         <v/>
       </c>
-      <c r="H15" s="139">
+      <c r="H15" s="141">
         <f>IF(C15=1,G15,G15-G14)</f>
         <v/>
       </c>
-      <c r="I15" s="139">
+      <c r="I15" s="141">
         <f>MAX(0,D15*'Premissas &amp; Cenários'!$B$44+H15*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J15" s="139">
+      <c r="J15" s="141">
         <f>I15*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K15" s="139">
+      <c r="K15" s="141">
         <f>MAX(0,I15-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L15" s="139">
+      <c r="L15" s="141">
         <f>MAX(0,D15*'Premissas &amp; Cenários'!$B$48+IF(AND(B15=2026,C15=1),0,H15*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M15" s="139">
+      <c r="M15" s="141">
         <f>L15*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N15" s="139">
+      <c r="N15" s="141">
         <f>J15+K15+M15</f>
         <v/>
       </c>
@@ -19877,7 +19912,7 @@
       <c r="A16" s="123" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="144">
+      <c r="B16" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A16-1)/4)</f>
         <v/>
       </c>
@@ -19885,47 +19920,47 @@
         <f>MOD(A16-1,4)+1</f>
         <v/>
       </c>
-      <c r="D16" s="140">
+      <c r="D16" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A16)</f>
         <v/>
       </c>
-      <c r="E16" s="139">
+      <c r="E16" s="141">
         <f>IF(C16=1,D16,E15+D16)</f>
         <v/>
       </c>
-      <c r="F16" s="140">
+      <c r="F16" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C16</f>
         <v/>
       </c>
-      <c r="G16" s="139">
+      <c r="G16" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E16-F16),0)</f>
         <v/>
       </c>
-      <c r="H16" s="139">
+      <c r="H16" s="141">
         <f>IF(C16=1,G16,G16-G15)</f>
         <v/>
       </c>
-      <c r="I16" s="139">
+      <c r="I16" s="141">
         <f>MAX(0,D16*'Premissas &amp; Cenários'!$B$44+H16*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J16" s="139">
+      <c r="J16" s="141">
         <f>I16*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K16" s="139">
+      <c r="K16" s="141">
         <f>MAX(0,I16-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L16" s="139">
+      <c r="L16" s="141">
         <f>MAX(0,D16*'Premissas &amp; Cenários'!$B$48+IF(AND(B16=2026,C16=1),0,H16*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M16" s="139">
+      <c r="M16" s="141">
         <f>L16*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N16" s="139">
+      <c r="N16" s="141">
         <f>J16+K16+M16</f>
         <v/>
       </c>
@@ -19934,7 +19969,7 @@
       <c r="A17" s="123" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="144">
+      <c r="B17" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A17-1)/4)</f>
         <v/>
       </c>
@@ -19942,47 +19977,47 @@
         <f>MOD(A17-1,4)+1</f>
         <v/>
       </c>
-      <c r="D17" s="140">
+      <c r="D17" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A17)</f>
         <v/>
       </c>
-      <c r="E17" s="139">
+      <c r="E17" s="141">
         <f>IF(C17=1,D17,E16+D17)</f>
         <v/>
       </c>
-      <c r="F17" s="140">
+      <c r="F17" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C17</f>
         <v/>
       </c>
-      <c r="G17" s="139">
+      <c r="G17" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E17-F17),0)</f>
         <v/>
       </c>
-      <c r="H17" s="139">
+      <c r="H17" s="141">
         <f>IF(C17=1,G17,G17-G16)</f>
         <v/>
       </c>
-      <c r="I17" s="139">
+      <c r="I17" s="141">
         <f>MAX(0,D17*'Premissas &amp; Cenários'!$B$44+H17*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J17" s="139">
+      <c r="J17" s="141">
         <f>I17*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K17" s="139">
+      <c r="K17" s="141">
         <f>MAX(0,I17-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L17" s="139">
+      <c r="L17" s="141">
         <f>MAX(0,D17*'Premissas &amp; Cenários'!$B$48+IF(AND(B17=2026,C17=1),0,H17*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M17" s="139">
+      <c r="M17" s="141">
         <f>L17*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N17" s="139">
+      <c r="N17" s="141">
         <f>J17+K17+M17</f>
         <v/>
       </c>
@@ -19991,7 +20026,7 @@
       <c r="A18" s="123" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="144">
+      <c r="B18" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A18-1)/4)</f>
         <v/>
       </c>
@@ -19999,47 +20034,47 @@
         <f>MOD(A18-1,4)+1</f>
         <v/>
       </c>
-      <c r="D18" s="140">
+      <c r="D18" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A18)</f>
         <v/>
       </c>
-      <c r="E18" s="139">
+      <c r="E18" s="141">
         <f>IF(C18=1,D18,E17+D18)</f>
         <v/>
       </c>
-      <c r="F18" s="140">
+      <c r="F18" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C18</f>
         <v/>
       </c>
-      <c r="G18" s="139">
+      <c r="G18" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E18-F18),0)</f>
         <v/>
       </c>
-      <c r="H18" s="139">
+      <c r="H18" s="141">
         <f>IF(C18=1,G18,G18-G17)</f>
         <v/>
       </c>
-      <c r="I18" s="139">
+      <c r="I18" s="141">
         <f>MAX(0,D18*'Premissas &amp; Cenários'!$B$44+H18*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J18" s="139">
+      <c r="J18" s="141">
         <f>I18*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K18" s="139">
+      <c r="K18" s="141">
         <f>MAX(0,I18-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L18" s="139">
+      <c r="L18" s="141">
         <f>MAX(0,D18*'Premissas &amp; Cenários'!$B$48+IF(AND(B18=2026,C18=1),0,H18*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M18" s="139">
+      <c r="M18" s="141">
         <f>L18*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N18" s="139">
+      <c r="N18" s="141">
         <f>J18+K18+M18</f>
         <v/>
       </c>
@@ -20048,7 +20083,7 @@
       <c r="A19" s="123" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="144">
+      <c r="B19" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A19-1)/4)</f>
         <v/>
       </c>
@@ -20056,47 +20091,47 @@
         <f>MOD(A19-1,4)+1</f>
         <v/>
       </c>
-      <c r="D19" s="140">
+      <c r="D19" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A19)</f>
         <v/>
       </c>
-      <c r="E19" s="139">
+      <c r="E19" s="141">
         <f>IF(C19=1,D19,E18+D19)</f>
         <v/>
       </c>
-      <c r="F19" s="140">
+      <c r="F19" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C19</f>
         <v/>
       </c>
-      <c r="G19" s="139">
+      <c r="G19" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E19-F19),0)</f>
         <v/>
       </c>
-      <c r="H19" s="139">
+      <c r="H19" s="141">
         <f>IF(C19=1,G19,G19-G18)</f>
         <v/>
       </c>
-      <c r="I19" s="139">
+      <c r="I19" s="141">
         <f>MAX(0,D19*'Premissas &amp; Cenários'!$B$44+H19*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J19" s="139">
+      <c r="J19" s="141">
         <f>I19*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K19" s="139">
+      <c r="K19" s="141">
         <f>MAX(0,I19-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L19" s="139">
+      <c r="L19" s="141">
         <f>MAX(0,D19*'Premissas &amp; Cenários'!$B$48+IF(AND(B19=2026,C19=1),0,H19*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M19" s="139">
+      <c r="M19" s="141">
         <f>L19*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N19" s="139">
+      <c r="N19" s="141">
         <f>J19+K19+M19</f>
         <v/>
       </c>
@@ -20105,7 +20140,7 @@
       <c r="A20" s="123" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="144">
+      <c r="B20" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A20-1)/4)</f>
         <v/>
       </c>
@@ -20113,47 +20148,47 @@
         <f>MOD(A20-1,4)+1</f>
         <v/>
       </c>
-      <c r="D20" s="140">
+      <c r="D20" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A20)</f>
         <v/>
       </c>
-      <c r="E20" s="139">
+      <c r="E20" s="141">
         <f>IF(C20=1,D20,E19+D20)</f>
         <v/>
       </c>
-      <c r="F20" s="140">
+      <c r="F20" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C20</f>
         <v/>
       </c>
-      <c r="G20" s="139">
+      <c r="G20" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E20-F20),0)</f>
         <v/>
       </c>
-      <c r="H20" s="139">
+      <c r="H20" s="141">
         <f>IF(C20=1,G20,G20-G19)</f>
         <v/>
       </c>
-      <c r="I20" s="139">
+      <c r="I20" s="141">
         <f>MAX(0,D20*'Premissas &amp; Cenários'!$B$44+H20*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J20" s="139">
+      <c r="J20" s="141">
         <f>I20*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K20" s="139">
+      <c r="K20" s="141">
         <f>MAX(0,I20-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L20" s="139">
+      <c r="L20" s="141">
         <f>MAX(0,D20*'Premissas &amp; Cenários'!$B$48+IF(AND(B20=2026,C20=1),0,H20*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M20" s="139">
+      <c r="M20" s="141">
         <f>L20*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N20" s="139">
+      <c r="N20" s="141">
         <f>J20+K20+M20</f>
         <v/>
       </c>
@@ -20162,7 +20197,7 @@
       <c r="A21" s="123" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="144">
+      <c r="B21" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A21-1)/4)</f>
         <v/>
       </c>
@@ -20170,47 +20205,47 @@
         <f>MOD(A21-1,4)+1</f>
         <v/>
       </c>
-      <c r="D21" s="140">
+      <c r="D21" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A21)</f>
         <v/>
       </c>
-      <c r="E21" s="139">
+      <c r="E21" s="141">
         <f>IF(C21=1,D21,E20+D21)</f>
         <v/>
       </c>
-      <c r="F21" s="140">
+      <c r="F21" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C21</f>
         <v/>
       </c>
-      <c r="G21" s="139">
+      <c r="G21" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E21-F21),0)</f>
         <v/>
       </c>
-      <c r="H21" s="139">
+      <c r="H21" s="141">
         <f>IF(C21=1,G21,G21-G20)</f>
         <v/>
       </c>
-      <c r="I21" s="139">
+      <c r="I21" s="141">
         <f>MAX(0,D21*'Premissas &amp; Cenários'!$B$44+H21*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J21" s="139">
+      <c r="J21" s="141">
         <f>I21*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K21" s="139">
+      <c r="K21" s="141">
         <f>MAX(0,I21-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L21" s="139">
+      <c r="L21" s="141">
         <f>MAX(0,D21*'Premissas &amp; Cenários'!$B$48+IF(AND(B21=2026,C21=1),0,H21*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M21" s="139">
+      <c r="M21" s="141">
         <f>L21*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N21" s="139">
+      <c r="N21" s="141">
         <f>J21+K21+M21</f>
         <v/>
       </c>
@@ -20219,7 +20254,7 @@
       <c r="A22" s="123" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="144">
+      <c r="B22" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A22-1)/4)</f>
         <v/>
       </c>
@@ -20227,47 +20262,47 @@
         <f>MOD(A22-1,4)+1</f>
         <v/>
       </c>
-      <c r="D22" s="140">
+      <c r="D22" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A22)</f>
         <v/>
       </c>
-      <c r="E22" s="139">
+      <c r="E22" s="141">
         <f>IF(C22=1,D22,E21+D22)</f>
         <v/>
       </c>
-      <c r="F22" s="140">
+      <c r="F22" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C22</f>
         <v/>
       </c>
-      <c r="G22" s="139">
+      <c r="G22" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E22-F22),0)</f>
         <v/>
       </c>
-      <c r="H22" s="139">
+      <c r="H22" s="141">
         <f>IF(C22=1,G22,G22-G21)</f>
         <v/>
       </c>
-      <c r="I22" s="139">
+      <c r="I22" s="141">
         <f>MAX(0,D22*'Premissas &amp; Cenários'!$B$44+H22*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J22" s="139">
+      <c r="J22" s="141">
         <f>I22*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K22" s="139">
+      <c r="K22" s="141">
         <f>MAX(0,I22-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L22" s="139">
+      <c r="L22" s="141">
         <f>MAX(0,D22*'Premissas &amp; Cenários'!$B$48+IF(AND(B22=2026,C22=1),0,H22*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M22" s="139">
+      <c r="M22" s="141">
         <f>L22*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N22" s="139">
+      <c r="N22" s="141">
         <f>J22+K22+M22</f>
         <v/>
       </c>
@@ -20276,7 +20311,7 @@
       <c r="A23" s="123" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="144">
+      <c r="B23" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A23-1)/4)</f>
         <v/>
       </c>
@@ -20284,47 +20319,47 @@
         <f>MOD(A23-1,4)+1</f>
         <v/>
       </c>
-      <c r="D23" s="140">
+      <c r="D23" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A23)</f>
         <v/>
       </c>
-      <c r="E23" s="139">
+      <c r="E23" s="141">
         <f>IF(C23=1,D23,E22+D23)</f>
         <v/>
       </c>
-      <c r="F23" s="140">
+      <c r="F23" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C23</f>
         <v/>
       </c>
-      <c r="G23" s="139">
+      <c r="G23" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E23-F23),0)</f>
         <v/>
       </c>
-      <c r="H23" s="139">
+      <c r="H23" s="141">
         <f>IF(C23=1,G23,G23-G22)</f>
         <v/>
       </c>
-      <c r="I23" s="139">
+      <c r="I23" s="141">
         <f>MAX(0,D23*'Premissas &amp; Cenários'!$B$44+H23*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J23" s="139">
+      <c r="J23" s="141">
         <f>I23*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K23" s="139">
+      <c r="K23" s="141">
         <f>MAX(0,I23-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L23" s="139">
+      <c r="L23" s="141">
         <f>MAX(0,D23*'Premissas &amp; Cenários'!$B$48+IF(AND(B23=2026,C23=1),0,H23*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M23" s="139">
+      <c r="M23" s="141">
         <f>L23*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N23" s="139">
+      <c r="N23" s="141">
         <f>J23+K23+M23</f>
         <v/>
       </c>
@@ -20333,7 +20368,7 @@
       <c r="A24" s="123" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="144">
+      <c r="B24" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A24-1)/4)</f>
         <v/>
       </c>
@@ -20341,47 +20376,47 @@
         <f>MOD(A24-1,4)+1</f>
         <v/>
       </c>
-      <c r="D24" s="140">
+      <c r="D24" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A24)</f>
         <v/>
       </c>
-      <c r="E24" s="139">
+      <c r="E24" s="141">
         <f>IF(C24=1,D24,E23+D24)</f>
         <v/>
       </c>
-      <c r="F24" s="140">
+      <c r="F24" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C24</f>
         <v/>
       </c>
-      <c r="G24" s="139">
+      <c r="G24" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E24-F24),0)</f>
         <v/>
       </c>
-      <c r="H24" s="139">
+      <c r="H24" s="141">
         <f>IF(C24=1,G24,G24-G23)</f>
         <v/>
       </c>
-      <c r="I24" s="139">
+      <c r="I24" s="141">
         <f>MAX(0,D24*'Premissas &amp; Cenários'!$B$44+H24*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J24" s="139">
+      <c r="J24" s="141">
         <f>I24*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K24" s="139">
+      <c r="K24" s="141">
         <f>MAX(0,I24-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L24" s="139">
+      <c r="L24" s="141">
         <f>MAX(0,D24*'Premissas &amp; Cenários'!$B$48+IF(AND(B24=2026,C24=1),0,H24*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M24" s="139">
+      <c r="M24" s="141">
         <f>L24*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N24" s="139">
+      <c r="N24" s="141">
         <f>J24+K24+M24</f>
         <v/>
       </c>
@@ -20390,7 +20425,7 @@
       <c r="A25" s="123" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="144">
+      <c r="B25" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A25-1)/4)</f>
         <v/>
       </c>
@@ -20398,47 +20433,47 @@
         <f>MOD(A25-1,4)+1</f>
         <v/>
       </c>
-      <c r="D25" s="140">
+      <c r="D25" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A25)</f>
         <v/>
       </c>
-      <c r="E25" s="139">
+      <c r="E25" s="141">
         <f>IF(C25=1,D25,E24+D25)</f>
         <v/>
       </c>
-      <c r="F25" s="140">
+      <c r="F25" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C25</f>
         <v/>
       </c>
-      <c r="G25" s="139">
+      <c r="G25" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E25-F25),0)</f>
         <v/>
       </c>
-      <c r="H25" s="139">
+      <c r="H25" s="141">
         <f>IF(C25=1,G25,G25-G24)</f>
         <v/>
       </c>
-      <c r="I25" s="139">
+      <c r="I25" s="141">
         <f>MAX(0,D25*'Premissas &amp; Cenários'!$B$44+H25*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J25" s="139">
+      <c r="J25" s="141">
         <f>I25*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K25" s="139">
+      <c r="K25" s="141">
         <f>MAX(0,I25-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L25" s="139">
+      <c r="L25" s="141">
         <f>MAX(0,D25*'Premissas &amp; Cenários'!$B$48+IF(AND(B25=2026,C25=1),0,H25*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M25" s="139">
+      <c r="M25" s="141">
         <f>L25*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N25" s="139">
+      <c r="N25" s="141">
         <f>J25+K25+M25</f>
         <v/>
       </c>
@@ -20447,7 +20482,7 @@
       <c r="A26" s="123" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="144">
+      <c r="B26" s="146">
         <f>'Premissas &amp; Cenários'!$B$50+INT((A26-1)/4)</f>
         <v/>
       </c>
@@ -20455,47 +20490,47 @@
         <f>MOD(A26-1,4)+1</f>
         <v/>
       </c>
-      <c r="D26" s="140">
+      <c r="D26" s="142">
         <f>SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$S$43:$S$102,A26)</f>
         <v/>
       </c>
-      <c r="E26" s="139">
+      <c r="E26" s="141">
         <f>IF(C26=1,D26,E25+D26)</f>
         <v/>
       </c>
-      <c r="F26" s="140">
+      <c r="F26" s="142">
         <f>'Premissas &amp; Cenários'!$B$106/4*C26</f>
         <v/>
       </c>
-      <c r="G26" s="139">
+      <c r="G26" s="141">
         <f>IF('Premissas &amp; Cenários'!$B$105="Sim",MAX(0,E26-F26),0)</f>
         <v/>
       </c>
-      <c r="H26" s="139">
+      <c r="H26" s="141">
         <f>IF(C26=1,G26,G26-G25)</f>
         <v/>
       </c>
-      <c r="I26" s="139">
+      <c r="I26" s="141">
         <f>MAX(0,D26*'Premissas &amp; Cenários'!$B$44+H26*'Premissas &amp; Cenários'!$B$44*'Premissas &amp; Cenários'!$B$107)</f>
         <v/>
       </c>
-      <c r="J26" s="139">
+      <c r="J26" s="141">
         <f>I26*'Premissas &amp; Cenários'!$B$45</f>
         <v/>
       </c>
-      <c r="K26" s="139">
+      <c r="K26" s="141">
         <f>MAX(0,I26-'Premissas &amp; Cenários'!$B$46)*'Premissas &amp; Cenários'!$B$47</f>
         <v/>
       </c>
-      <c r="L26" s="139">
+      <c r="L26" s="141">
         <f>MAX(0,D26*'Premissas &amp; Cenários'!$B$48+IF(AND(B26=2026,C26=1),0,H26*'Premissas &amp; Cenários'!$B$48*'Premissas &amp; Cenários'!$B$107))</f>
         <v/>
       </c>
-      <c r="M26" s="139">
+      <c r="M26" s="141">
         <f>L26*'Premissas &amp; Cenários'!$B$49</f>
         <v/>
       </c>
-      <c r="N26" s="139">
+      <c r="N26" s="141">
         <f>J26+K26+M26</f>
         <v/>
       </c>
@@ -20506,35 +20541,35 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="D27" s="141">
+      <c r="D27" s="143">
         <f>SUM(D7:D26)</f>
         <v/>
       </c>
-      <c r="H27" s="141">
+      <c r="H27" s="143">
         <f>SUM(H7:H26)</f>
         <v/>
       </c>
-      <c r="I27" s="141">
+      <c r="I27" s="143">
         <f>SUM(I7:I26)</f>
         <v/>
       </c>
-      <c r="J27" s="141">
+      <c r="J27" s="143">
         <f>SUM(J7:J26)</f>
         <v/>
       </c>
-      <c r="K27" s="141">
+      <c r="K27" s="143">
         <f>SUM(K7:K26)</f>
         <v/>
       </c>
-      <c r="L27" s="141">
+      <c r="L27" s="143">
         <f>SUM(L7:L26)</f>
         <v/>
       </c>
-      <c r="M27" s="141">
+      <c r="M27" s="143">
         <f>SUM(M7:M26)</f>
         <v/>
       </c>
-      <c r="N27" s="141">
+      <c r="N27" s="143">
         <f>SUM(N7:N26)</f>
         <v/>
       </c>
@@ -20545,7 +20580,7 @@
           <t>Check receita</t>
         </is>
       </c>
-      <c r="D28" s="141">
+      <c r="D28" s="143">
         <f>D27-Fluxo_Incorporacao!$B$103</f>
         <v/>
       </c>
@@ -20580,18 +20615,18 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="142" t="inlineStr">
+      <c r="A1" s="144" t="inlineStr">
         <is>
           <t>Comparativo — regime regular × RET de transição (art. 485)</t>
         </is>
       </c>
-      <c r="B1" s="143" t="n"/>
-      <c r="C1" s="143" t="n"/>
-      <c r="D1" s="143" t="n"/>
-      <c r="E1" s="143" t="n"/>
-      <c r="F1" s="143" t="n"/>
-      <c r="G1" s="143" t="n"/>
-      <c r="H1" s="143" t="n"/>
+      <c r="B1" s="145" t="n"/>
+      <c r="C1" s="145" t="n"/>
+      <c r="D1" s="145" t="n"/>
+      <c r="E1" s="145" t="n"/>
+      <c r="F1" s="145" t="n"/>
+      <c r="G1" s="145" t="n"/>
+      <c r="H1" s="145" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -20614,23 +20649,23 @@
           <t>Rubrica</t>
         </is>
       </c>
-      <c r="B6" s="127">
+      <c r="B6" s="147">
         <f>'Premissas &amp; Cenários'!$B$50+0</f>
         <v/>
       </c>
-      <c r="C6" s="127">
+      <c r="C6" s="147">
         <f>'Premissas &amp; Cenários'!$B$50+1</f>
         <v/>
       </c>
-      <c r="D6" s="127">
+      <c r="D6" s="147">
         <f>'Premissas &amp; Cenários'!$B$50+2</f>
         <v/>
       </c>
-      <c r="E6" s="127">
+      <c r="E6" s="147">
         <f>'Premissas &amp; Cenários'!$B$50+3</f>
         <v/>
       </c>
-      <c r="F6" s="127">
+      <c r="F6" s="147">
         <f>'Premissas &amp; Cenários'!$B$50+4</f>
         <v/>
       </c>
@@ -20651,31 +20686,31 @@
           <t>Recebimentos (VGV tributável)</t>
         </is>
       </c>
-      <c r="B7" s="140">
+      <c r="B7" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$N$43:$N$102,B$6),0)</f>
         <v/>
       </c>
-      <c r="C7" s="140">
+      <c r="C7" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$N$43:$N$102,C$6),0)</f>
         <v/>
       </c>
-      <c r="D7" s="140">
+      <c r="D7" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$N$43:$N$102,D$6),0)</f>
         <v/>
       </c>
-      <c r="E7" s="140">
+      <c r="E7" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$N$43:$N$102,E$6),0)</f>
         <v/>
       </c>
-      <c r="F7" s="140">
+      <c r="F7" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$B$43:$B$102,Fluxo_Incorporacao!$N$43:$N$102,F$6),0)</f>
         <v/>
       </c>
-      <c r="G7" s="139">
+      <c r="G7" s="141">
         <f>SUM(B7:F7)</f>
         <v/>
       </c>
-      <c r="H7" s="139">
+      <c r="H7" s="141">
         <f>B7/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C7/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D7/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E7/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F7/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20701,31 +20736,31 @@
           <t>PIS/Cofins cumulativo (2026)</t>
         </is>
       </c>
-      <c r="B10" s="140">
+      <c r="B10" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$R$43:$R$102,Fluxo_Incorporacao!$N$43:$N$102,B$6),0)</f>
         <v/>
       </c>
-      <c r="C10" s="140">
+      <c r="C10" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$R$43:$R$102,Fluxo_Incorporacao!$N$43:$N$102,C$6),0)</f>
         <v/>
       </c>
-      <c r="D10" s="140">
+      <c r="D10" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$R$43:$R$102,Fluxo_Incorporacao!$N$43:$N$102,D$6),0)</f>
         <v/>
       </c>
-      <c r="E10" s="140">
+      <c r="E10" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$R$43:$R$102,Fluxo_Incorporacao!$N$43:$N$102,E$6),0)</f>
         <v/>
       </c>
-      <c r="F10" s="140">
+      <c r="F10" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$R$43:$R$102,Fluxo_Incorporacao!$N$43:$N$102,F$6),0)</f>
         <v/>
       </c>
-      <c r="G10" s="139">
+      <c r="G10" s="141">
         <f>SUM(B10:F10)</f>
         <v/>
       </c>
-      <c r="H10" s="139">
+      <c r="H10" s="141">
         <f>B10/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C10/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D10/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E10/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F10/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20736,31 +20771,31 @@
           <t>IBS + CBS recolhido (após créditos)</t>
         </is>
       </c>
-      <c r="B11" s="140">
+      <c r="B11" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$J$43:$J$102,Fluxo_Incorporacao!$N$43:$N$102,B$6),0)</f>
         <v/>
       </c>
-      <c r="C11" s="140">
+      <c r="C11" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$J$43:$J$102,Fluxo_Incorporacao!$N$43:$N$102,C$6),0)</f>
         <v/>
       </c>
-      <c r="D11" s="140">
+      <c r="D11" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$J$43:$J$102,Fluxo_Incorporacao!$N$43:$N$102,D$6),0)</f>
         <v/>
       </c>
-      <c r="E11" s="140">
+      <c r="E11" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$J$43:$J$102,Fluxo_Incorporacao!$N$43:$N$102,E$6),0)</f>
         <v/>
       </c>
-      <c r="F11" s="140">
+      <c r="F11" s="142">
         <f>IFERROR(SUMIFS(Fluxo_Incorporacao!$J$43:$J$102,Fluxo_Incorporacao!$N$43:$N$102,F$6),0)</f>
         <v/>
       </c>
-      <c r="G11" s="139">
+      <c r="G11" s="141">
         <f>SUM(B11:F11)</f>
         <v/>
       </c>
-      <c r="H11" s="139">
+      <c r="H11" s="141">
         <f>B11/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C11/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D11/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E11/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F11/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20771,31 +20806,31 @@
           <t>IRPJ + CSLL (trimestral, LC 224)</t>
         </is>
       </c>
-      <c r="B12" s="140">
+      <c r="B12" s="142">
         <f>IFERROR(SUMIFS('IRPJ_CSLL Trimestral'!$N$7:$N$26,'IRPJ_CSLL Trimestral'!$B$7:$B$26,B$6),0)</f>
         <v/>
       </c>
-      <c r="C12" s="140">
+      <c r="C12" s="142">
         <f>IFERROR(SUMIFS('IRPJ_CSLL Trimestral'!$N$7:$N$26,'IRPJ_CSLL Trimestral'!$B$7:$B$26,C$6),0)</f>
         <v/>
       </c>
-      <c r="D12" s="140">
+      <c r="D12" s="142">
         <f>IFERROR(SUMIFS('IRPJ_CSLL Trimestral'!$N$7:$N$26,'IRPJ_CSLL Trimestral'!$B$7:$B$26,D$6),0)</f>
         <v/>
       </c>
-      <c r="E12" s="140">
+      <c r="E12" s="142">
         <f>IFERROR(SUMIFS('IRPJ_CSLL Trimestral'!$N$7:$N$26,'IRPJ_CSLL Trimestral'!$B$7:$B$26,E$6),0)</f>
         <v/>
       </c>
-      <c r="F12" s="140">
+      <c r="F12" s="142">
         <f>IFERROR(SUMIFS('IRPJ_CSLL Trimestral'!$N$7:$N$26,'IRPJ_CSLL Trimestral'!$B$7:$B$26,F$6),0)</f>
         <v/>
       </c>
-      <c r="G12" s="139">
+      <c r="G12" s="141">
         <f>SUM(B12:F12)</f>
         <v/>
       </c>
-      <c r="H12" s="139">
+      <c r="H12" s="141">
         <f>B12/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C12/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D12/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E12/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F12/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20806,31 +20841,31 @@
           <t>Total — regime regular</t>
         </is>
       </c>
-      <c r="B13" s="141">
+      <c r="B13" s="143">
         <f>SUM(B10:B12)</f>
         <v/>
       </c>
-      <c r="C13" s="141">
+      <c r="C13" s="143">
         <f>SUM(C10:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="141">
+      <c r="D13" s="143">
         <f>SUM(D10:D12)</f>
         <v/>
       </c>
-      <c r="E13" s="141">
+      <c r="E13" s="143">
         <f>SUM(E10:E12)</f>
         <v/>
       </c>
-      <c r="F13" s="141">
+      <c r="F13" s="143">
         <f>SUM(F10:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="141">
+      <c r="G13" s="143">
         <f>SUM(B13:F13)</f>
         <v/>
       </c>
-      <c r="H13" s="141">
+      <c r="H13" s="143">
         <f>B13/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C13/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D13/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E13/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F13/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20887,31 +20922,31 @@
           <t>RET — IRPJ + CSLL</t>
         </is>
       </c>
-      <c r="B17" s="139">
+      <c r="B17" s="141">
         <f>B7*'Premissas &amp; Cenários'!$B$113</f>
         <v/>
       </c>
-      <c r="C17" s="139">
+      <c r="C17" s="141">
         <f>C7*'Premissas &amp; Cenários'!$B$113</f>
         <v/>
       </c>
-      <c r="D17" s="139">
+      <c r="D17" s="141">
         <f>D7*'Premissas &amp; Cenários'!$B$113</f>
         <v/>
       </c>
-      <c r="E17" s="139">
+      <c r="E17" s="141">
         <f>E7*'Premissas &amp; Cenários'!$B$113</f>
         <v/>
       </c>
-      <c r="F17" s="139">
+      <c r="F17" s="141">
         <f>F7*'Premissas &amp; Cenários'!$B$113</f>
         <v/>
       </c>
-      <c r="G17" s="139">
+      <c r="G17" s="141">
         <f>SUM(B17:F17)</f>
         <v/>
       </c>
-      <c r="H17" s="139">
+      <c r="H17" s="141">
         <f>B17/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C17/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D17/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E17/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F17/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20922,31 +20957,31 @@
           <t>RET — PIS/Cofins (2026) e IBS + CBS (2027 em diante)</t>
         </is>
       </c>
-      <c r="B18" s="139">
+      <c r="B18" s="141">
         <f>B7*'Premissas &amp; Cenários'!$B$114</f>
         <v/>
       </c>
-      <c r="C18" s="139">
+      <c r="C18" s="141">
         <f>C7*'Premissas &amp; Cenários'!$B$114</f>
         <v/>
       </c>
-      <c r="D18" s="139">
+      <c r="D18" s="141">
         <f>D7*'Premissas &amp; Cenários'!$B$114</f>
         <v/>
       </c>
-      <c r="E18" s="139">
+      <c r="E18" s="141">
         <f>E7*'Premissas &amp; Cenários'!$B$114</f>
         <v/>
       </c>
-      <c r="F18" s="139">
+      <c r="F18" s="141">
         <f>F7*'Premissas &amp; Cenários'!$B$114</f>
         <v/>
       </c>
-      <c r="G18" s="139">
+      <c r="G18" s="141">
         <f>SUM(B18:F18)</f>
         <v/>
       </c>
-      <c r="H18" s="139">
+      <c r="H18" s="141">
         <f>B18/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C18/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D18/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E18/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F18/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -20957,31 +20992,31 @@
           <t>Total — RET</t>
         </is>
       </c>
-      <c r="B19" s="141">
+      <c r="B19" s="143">
         <f>B17+B18</f>
         <v/>
       </c>
-      <c r="C19" s="141">
+      <c r="C19" s="143">
         <f>C17+C18</f>
         <v/>
       </c>
-      <c r="D19" s="141">
+      <c r="D19" s="143">
         <f>D17+D18</f>
         <v/>
       </c>
-      <c r="E19" s="141">
+      <c r="E19" s="143">
         <f>E17+E18</f>
         <v/>
       </c>
-      <c r="F19" s="141">
+      <c r="F19" s="143">
         <f>F17+F18</f>
         <v/>
       </c>
-      <c r="G19" s="141">
+      <c r="G19" s="143">
         <f>SUM(B19:F19)</f>
         <v/>
       </c>
-      <c r="H19" s="141">
+      <c r="H19" s="143">
         <f>B19/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C19/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D19/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E19/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F19/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -21024,31 +21059,31 @@
           <t>Diferença: regime regular − RET (positivo = RET paga menos)</t>
         </is>
       </c>
-      <c r="B22" s="141">
+      <c r="B22" s="143">
         <f>B13-B19</f>
         <v/>
       </c>
-      <c r="C22" s="141">
+      <c r="C22" s="143">
         <f>C13-C19</f>
         <v/>
       </c>
-      <c r="D22" s="141">
+      <c r="D22" s="143">
         <f>D13-D19</f>
         <v/>
       </c>
-      <c r="E22" s="141">
+      <c r="E22" s="143">
         <f>E13-E19</f>
         <v/>
       </c>
-      <c r="F22" s="141">
+      <c r="F22" s="143">
         <f>F13-F19</f>
         <v/>
       </c>
-      <c r="G22" s="141">
+      <c r="G22" s="143">
         <f>SUM(B22:F22)</f>
         <v/>
       </c>
-      <c r="H22" s="141">
+      <c r="H22" s="143">
         <f>B22/(1+'Premissas &amp; Cenários'!$B$115)^0.5+C22/(1+'Premissas &amp; Cenários'!$B$115)^1.5+D22/(1+'Premissas &amp; Cenários'!$B$115)^2.5+E22/(1+'Premissas &amp; Cenários'!$B$115)^3.5+F22/(1+'Premissas &amp; Cenários'!$B$115)^4.5</f>
         <v/>
       </c>
@@ -21070,7 +21105,7 @@
           <t>Saldo credor de IBS/CBS ao fim do ciclo (regime regular; não incluído acima)</t>
         </is>
       </c>
-      <c r="G24" s="140">
+      <c r="G24" s="142">
         <f>Fluxo_Incorporacao!$K$102</f>
         <v/>
       </c>
@@ -21840,13 +21875,13 @@
       </c>
     </row>
     <row r="13" ht="38.25" customHeight="1">
-      <c r="A13" s="98" t="n">
+      <c r="A13" s="148" t="n">
         <v>2026</v>
       </c>
-      <c r="B13" s="145" t="n">
+      <c r="B13" s="149" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="C13" s="145" t="n">
+      <c r="C13" s="149" t="n">
         <v>0.001</v>
       </c>
       <c r="D13" s="99" t="n">
@@ -21856,11 +21891,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F13" s="146">
+      <c r="F13" s="150">
         <f>IF(OR(B13="",C13=""),"",IFERROR((B13+C13)*(1-E13),0))</f>
         <v/>
       </c>
-      <c r="G13" s="146">
+      <c r="G13" s="150">
         <f>IF(F13="","",IF(J13="Sim",0,F13))</f>
         <v/>
       </c>
@@ -21873,29 +21908,29 @@
         <f>IF(AND(B13&lt;&gt;"",C13&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J13" s="130" t="inlineStr">
+      <c r="J13" s="151" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="K13" s="147">
+      <c r="K13" s="152">
         <f>'Premissas &amp; Cenários'!$B$110</f>
         <v/>
       </c>
-      <c r="L13" s="126">
+      <c r="L13" s="153">
         <f>IF(J13="Sim",0,IFERROR(F13/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="25.5" customHeight="1">
-      <c r="A14" s="104" t="n">
+      <c r="A14" s="154" t="n">
         <v>2027</v>
       </c>
-      <c r="B14" s="148">
+      <c r="B14" s="155">
         <f>'Premissas &amp; Cenários'!$B$108-0.001</f>
         <v/>
       </c>
-      <c r="C14" s="145" t="n">
+      <c r="C14" s="156" t="n">
         <v>0.001</v>
       </c>
       <c r="D14" s="106" t="n">
@@ -21905,11 +21940,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F14" s="149">
+      <c r="F14" s="157">
         <f>IF(OR(B14="",C14=""),"",IFERROR((B14+C14)*(1-E14),0))</f>
         <v/>
       </c>
-      <c r="G14" s="149">
+      <c r="G14" s="157">
         <f>IF(F14="","",IF(J14="Sim",0,F14))</f>
         <v/>
       </c>
@@ -21922,28 +21957,28 @@
         <f>IF(AND(B14&lt;&gt;"",C14&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J14" s="130" t="inlineStr">
+      <c r="J14" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K14" s="132" t="n">
+      <c r="K14" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="126">
+      <c r="L14" s="160">
         <f>IF(J14="Sim",0,IFERROR(F14/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="25.5" customHeight="1">
-      <c r="A15" s="104" t="n">
+      <c r="A15" s="154" t="n">
         <v>2028</v>
       </c>
-      <c r="B15" s="148">
+      <c r="B15" s="155">
         <f>'Premissas &amp; Cenários'!$B$108-0.001</f>
         <v/>
       </c>
-      <c r="C15" s="145" t="n">
+      <c r="C15" s="156" t="n">
         <v>0.001</v>
       </c>
       <c r="D15" s="106" t="n">
@@ -21953,11 +21988,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F15" s="149">
+      <c r="F15" s="157">
         <f>IF(OR(B15="",C15=""),"",IFERROR((B15+C15)*(1-E15),0))</f>
         <v/>
       </c>
-      <c r="G15" s="149">
+      <c r="G15" s="157">
         <f>IF(F15="","",IF(J15="Sim",0,F15))</f>
         <v/>
       </c>
@@ -21970,28 +22005,28 @@
         <f>IF(AND(B15&lt;&gt;"",C15&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J15" s="130" t="inlineStr">
+      <c r="J15" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K15" s="132" t="n">
+      <c r="K15" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="126">
+      <c r="L15" s="160">
         <f>IF(J15="Sim",0,IFERROR(F15/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="38.25" customHeight="1">
-      <c r="A16" s="104" t="n">
+      <c r="A16" s="154" t="n">
         <v>2029</v>
       </c>
-      <c r="B16" s="148">
+      <c r="B16" s="155">
         <f>'Premissas &amp; Cenários'!$B$108</f>
         <v/>
       </c>
-      <c r="C16" s="148">
+      <c r="C16" s="155">
         <f>'Premissas &amp; Cenários'!$B$109*0.1</f>
         <v/>
       </c>
@@ -22002,11 +22037,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F16" s="149">
+      <c r="F16" s="157">
         <f>IF(OR(B16="",C16=""),"",IFERROR((B16+C16)*(1-E16),0))</f>
         <v/>
       </c>
-      <c r="G16" s="149">
+      <c r="G16" s="157">
         <f>IF(F16="","",IF(J16="Sim",0,F16))</f>
         <v/>
       </c>
@@ -22019,28 +22054,28 @@
         <f>IF(AND(B16&lt;&gt;"",C16&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J16" s="130" t="inlineStr">
+      <c r="J16" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K16" s="132" t="n">
+      <c r="K16" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="126">
+      <c r="L16" s="160">
         <f>IF(J16="Sim",0,IFERROR(F16/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="25.5" customHeight="1">
-      <c r="A17" s="104" t="n">
+      <c r="A17" s="154" t="n">
         <v>2030</v>
       </c>
-      <c r="B17" s="148">
+      <c r="B17" s="155">
         <f>'Premissas &amp; Cenários'!$B$108</f>
         <v/>
       </c>
-      <c r="C17" s="148">
+      <c r="C17" s="155">
         <f>'Premissas &amp; Cenários'!$B$109*0.2</f>
         <v/>
       </c>
@@ -22051,11 +22086,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F17" s="149">
+      <c r="F17" s="157">
         <f>IF(OR(B17="",C17=""),"",IFERROR((B17+C17)*(1-E17),0))</f>
         <v/>
       </c>
-      <c r="G17" s="149">
+      <c r="G17" s="157">
         <f>IF(F17="","",IF(J17="Sim",0,F17))</f>
         <v/>
       </c>
@@ -22068,28 +22103,28 @@
         <f>IF(AND(B17&lt;&gt;"",C17&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J17" s="130" t="inlineStr">
+      <c r="J17" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K17" s="132" t="n">
+      <c r="K17" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="126">
+      <c r="L17" s="160">
         <f>IF(J17="Sim",0,IFERROR(F17/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="25.5" customHeight="1">
-      <c r="A18" s="104" t="n">
+      <c r="A18" s="154" t="n">
         <v>2031</v>
       </c>
-      <c r="B18" s="148">
+      <c r="B18" s="155">
         <f>'Premissas &amp; Cenários'!$B$108</f>
         <v/>
       </c>
-      <c r="C18" s="148">
+      <c r="C18" s="155">
         <f>'Premissas &amp; Cenários'!$B$109*0.3</f>
         <v/>
       </c>
@@ -22100,11 +22135,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F18" s="149">
+      <c r="F18" s="157">
         <f>IF(OR(B18="",C18=""),"",IFERROR((B18+C18)*(1-E18),0))</f>
         <v/>
       </c>
-      <c r="G18" s="149">
+      <c r="G18" s="157">
         <f>IF(F18="","",IF(J18="Sim",0,F18))</f>
         <v/>
       </c>
@@ -22117,28 +22152,28 @@
         <f>IF(AND(B18&lt;&gt;"",C18&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J18" s="130" t="inlineStr">
+      <c r="J18" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K18" s="132" t="n">
+      <c r="K18" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L18" s="126">
+      <c r="L18" s="160">
         <f>IF(J18="Sim",0,IFERROR(F18/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="25.5" customHeight="1">
-      <c r="A19" s="104" t="n">
+      <c r="A19" s="154" t="n">
         <v>2032</v>
       </c>
-      <c r="B19" s="148">
+      <c r="B19" s="155">
         <f>'Premissas &amp; Cenários'!$B$108</f>
         <v/>
       </c>
-      <c r="C19" s="148">
+      <c r="C19" s="155">
         <f>'Premissas &amp; Cenários'!$B$109*0.4</f>
         <v/>
       </c>
@@ -22149,11 +22184,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F19" s="149">
+      <c r="F19" s="157">
         <f>IF(OR(B19="",C19=""),"",IFERROR((B19+C19)*(1-E19),0))</f>
         <v/>
       </c>
-      <c r="G19" s="149">
+      <c r="G19" s="157">
         <f>IF(F19="","",IF(J19="Sim",0,F19))</f>
         <v/>
       </c>
@@ -22166,28 +22201,28 @@
         <f>IF(AND(B19&lt;&gt;"",C19&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J19" s="130" t="inlineStr">
+      <c r="J19" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K19" s="132" t="n">
+      <c r="K19" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L19" s="126">
+      <c r="L19" s="160">
         <f>IF(J19="Sim",0,IFERROR(F19/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="38.25" customHeight="1">
-      <c r="A20" s="104" t="n">
+      <c r="A20" s="154" t="n">
         <v>2033</v>
       </c>
-      <c r="B20" s="148">
+      <c r="B20" s="155">
         <f>'Premissas &amp; Cenários'!$B$108</f>
         <v/>
       </c>
-      <c r="C20" s="148">
+      <c r="C20" s="155">
         <f>'Premissas &amp; Cenários'!$B$109</f>
         <v/>
       </c>
@@ -22198,11 +22233,11 @@
         <f>'Premissas &amp; Cenários'!$B$34</f>
         <v/>
       </c>
-      <c r="F20" s="149">
+      <c r="F20" s="157">
         <f>IF(OR(B20="",C20=""),"",IFERROR((B20+C20)*(1-E20),0))</f>
         <v/>
       </c>
-      <c r="G20" s="149">
+      <c r="G20" s="157">
         <f>IF(F20="","",IF(J20="Sim",0,F20))</f>
         <v/>
       </c>
@@ -22215,15 +22250,15 @@
         <f>IF(AND(B20&lt;&gt;"",C20&lt;&gt;""),"OK","PENDENTE")</f>
         <v/>
       </c>
-      <c r="J20" s="130" t="inlineStr">
+      <c r="J20" s="158" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="K20" s="132" t="n">
+      <c r="K20" s="159" t="n">
         <v>0</v>
       </c>
-      <c r="L20" s="126">
+      <c r="L20" s="160">
         <f>IF(J20="Sim",0,IFERROR(F20/'Premissas &amp; Cenários'!$B$35,0))</f>
         <v/>
       </c>

</xml_diff>